<commit_message>
feat: add transition underwriting and pilots
- separate enterprise and project result bases
- add investor and deal screens with KR/JP dry runs
- enforce internal release gates through CI and validation docs
</commit_message>
<xml_diff>
--- a/config/calibration.xlsx
+++ b/config/calibration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -665,37 +665,76 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>feedstock</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Naphtha/circular-feed spread volatility — route-specific market series not yet ingested; IEA feedstock-cost sensitivity anchor</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>#axiom-linear-cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>capex</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>0.15</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C8" t="n">
         <v>0.1</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>-0.03</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>assumed</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>K07 밴드 620–830 (±15% around 700); μ=학습률 8%/doubling 근사 (capex_h2dri_references.csv)</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>#axiom-linear-cost</t>
         </is>
@@ -712,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,6 +1007,150 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>#axiom-linear-cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>feedstock</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>carbon</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Naphtha-carbon common fossil cycle; matched time series not yet ingested</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>#claim-policy-repricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>feedstock</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>elec</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Energy-complex common factor; matched time series not yet ingested</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>#axiom-linear-cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>feedstock</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>h2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Alternative-feed and hydrogen price co-movement uncalibrated — base 0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>#axiom-linear-cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>feedstock</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>capex</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>assumed</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No empirical anchor — base 0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>#axiom-linear-cost</t>
         </is>
@@ -984,7 +1167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1042,11 +1225,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>p_bind</t>
+          <t>k</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1055,23 +1238,23 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>넷제로 예산 구속확률 — 수준에만 진입 anatomy 불진입 (A2)</t>
+          <t>ATM 옵션가치 선형화 상수 (≈0.4σB); LSM이 근사 없이 같은 대상 계산</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>#axiom-budget-binds</t>
+          <t>#claim-lambda-invariance</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>fx_usdkrw</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4</v>
+        <v>1300</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1080,23 +1263,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ATM 옵션가치 선형화 상수 (≈0.4σB); LSM이 근사 없이 같은 대상 계산</t>
+          <t>2026 근사 환율 — ingest USD 병기용</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>#claim-lambda-invariance</t>
+          <t>#ledger-logic</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fx_usdkrw</t>
+          <t>fx_usdjpy</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1300</v>
+        <v>150</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1117,73 +1300,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fx_usdjpy</t>
+          <t>carbon_base_kr</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150</v>
+        <v>14.93</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>assumed</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026 근사 환율 — ingest USD 병기용</t>
+          <t>KAU 2026-06-30 종가 (ICAP 레퍼런스; outputs/reference_prices.json 연단위 대조) — 시나리오화 시 이 행을 시나리오가 대체</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>#ledger-logic</t>
+          <t>#claim-policy-repricing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>carbon_base_kr</t>
+          <t>carbon_base_jp</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14.93</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>banded</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KAU 2026-06-30 종가 (ICAP 레퍼런스; outputs/reference_prices.json 연단위 대조) — 시나리오화 시 이 행을 시나리오가 대체</t>
+          <t>GX-ETS 초기 시세 근사 (ICAP 2025; price_parameters.csv P07)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
-        <is>
-          <t>#claim-policy-repricing</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>carbon_base_jp</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>banded</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>GX-ETS 초기 시세 근사 (ICAP 2025; price_parameters.csv P07)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
         <is>
           <t>#claim-policy-repricing</t>
         </is>
@@ -1200,7 +1358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1253,214 +1411,259 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>n_paths</t>
+          <t>mu_anchor_years</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4000</v>
+        <v>15</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Monte Carlo 경로 수</t>
+          <t>μ_carbon 시나리오 앵커 지평 — carbon_reform 개입 시 drift 재산정에 사용</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>horizon_years</t>
+          <t>tau_exercise_threshold</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>0.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>시뮬레이션 지평 (~2060 reline 윈도우)</t>
+          <t>τ* 정의: 경로 행사비율이 이 값에 도달하는 첫 해 (p50) — 조건부 평균의 선택편의 회피</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>basis_degree</t>
+          <t>n_paths</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4000</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LSM 회귀 basis 다항 차수</t>
+          <t>Monte Carlo 경로 수</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>lambda_grid_lo</t>
+          <t>horizon_years</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.15</v>
+        <v>35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>s05 λ×p_bind 격자</t>
+          <t>시뮬레이션 지평 (~2060 reline 윈도우)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lambda_grid_hi</t>
+          <t>basis_degree</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LSM 회귀 basis 다항 차수</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lambda_grid_n</t>
+          <t>lambda_grid_lo</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
+        <v>0.15</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>s05 λ×p_bind 격자</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>p_bind_grid_lo</t>
+          <t>lambda_grid_hi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.25</v>
+        <v>0.65</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>p_bind_grid_hi</t>
+          <t>lambda_grid_n</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.95</v>
+        <v>6</v>
       </c>
       <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>p_bind_grid_n</t>
+          <t>p_bind_grid_lo</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>0.25</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>n_band_draws</t>
+          <t>p_bind_grid_hi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>200</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>s05 share envelope: σ·ρ band 내 draw 수 — 분산 분해 A1 #axiom-variance-not-mean</t>
-        </is>
-      </c>
+        <v>0.95</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sigma_linearity_n</t>
+          <t>p_bind_grid_n</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>s03 σ 스케일 격자 점수 (R² 체크)</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>p_bind_in_exercise</t>
+          <t>n_band_draws</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>실험 플래그(R5): p_bind를 행사정책에 투입 — 기본 off, LEDGER 자동 표기</t>
+          <t>s05 share envelope: σ·ρ band 내 draw 수 — 분산 분해 A1 #axiom-variance-not-mean</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lambda_k_carbon</t>
+          <t>sigma_linearity_n</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5</v>
+        <v>7</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>s05 driver별 λ_k 감응도 모듈 (R1 대응) — 시스템적 점프리스크 가중</t>
+          <t>s03 σ 스케일 격자 점수 (R² 체크)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lambda_k_h2</t>
+          <t>p_bind_in_exercise</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>부분 분산가능 기술리스크</t>
+          <t>실험 플래그(R5): p_bind를 행사정책에 투입 — 기본 off, LEDGER 자동 표기</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lambda_k_elec</t>
+          <t>lambda_k_carbon</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
+        <v>0.5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>s05 driver별 λ_k 감응도 모듈 (R1 대응) — 시스템적 점프리스크 가중</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>lambda_k_h2</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>부분 분산가능 기술리스크</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>lambda_k_elec</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>lambda_k_feedstock</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>commodity/feedstock exposure — provisional systematic-risk weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>lambda_k_capex</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B22" t="n">
         <v>0.3</v>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1473,7 +1676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1504,6 +1707,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>factor</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>anchor_note</t>
         </is>
       </c>
@@ -1511,7 +1719,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>carbon</t>
+          <t>carbon_kr</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1530,6 +1738,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>domestic</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>현상유지 — KAU 얇은 시장 관성 (#claim-policy-repricing); 예산 비구속</t>
         </is>
       </c>
@@ -1537,7 +1750,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>carbon</t>
+          <t>carbon_kr</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1556,14 +1769,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MSR 도입 + 이월제한 개혁 — 시장안정예비 (#claim-policy-repricing)</t>
+          <t>domestic</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MSR 도입 + 이월제한 개혁 (#claim-policy-repricing #axiom-budget-binds)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>carbon</t>
+          <t>carbon_kr</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1582,7 +1800,105 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CBAM 연계·EUA 수렴 (#claim-policy-repricing); EUA-KAU 스프레드 앵커링 필요 (R2)</t>
+          <t>cbam_common</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CBAM 연계·EUA 수렴 (#claim-policy-repricing #axiom-budget-binds); EUA-KAU 스프레드 앵커링 필요 (R2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>carbon_jp</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SQ</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>domestic</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>GX-ETS 초기 저가 관성 (assumed; ICAP/METI) — 비구속</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>carbon_jp</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GX_COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>domestic</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>GX-ETS 의무화 2단계 + 옥션 (assumed; #axiom-budget-binds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>carbon_jp</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>85</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>cbam_common</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CBAM 연계·EUA 수렴 (assumed; #axiom-budget-binds); KR과 공통요인</t>
         </is>
       </c>
     </row>

</xml_diff>